<commit_message>
versão com a automação de medição pronta
</commit_message>
<xml_diff>
--- a/testes/medicao_blueez_teste.xlsx
+++ b/testes/medicao_blueez_teste.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\Controller_Automacoes\Gerenciador_Automacoes\testes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0A0F2B-C827-4CB0-BDE5-ED7B815CA613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5382CF4B-0D37-4BE6-B5DA-98F685BAB40B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>empresa</t>
   </si>
@@ -83,22 +83,25 @@
     <t>Gustavo@1025</t>
   </si>
   <si>
-    <t xml:space="preserve">MEGA INFRA SOLUCOES EM INFRAESTRUTURA </t>
-  </si>
-  <si>
-    <t>CAIS NETWORK COM E SERVICOS DE TEL E INFORMATICA LTDA ME</t>
-  </si>
-  <si>
-    <t>07.798.532/0001-65</t>
-  </si>
-  <si>
-    <t>6949</t>
-  </si>
-  <si>
-    <t>BOLETO CAIS 6.000,00</t>
-  </si>
-  <si>
-    <t>NF CAIS 6.000,00 6949</t>
+    <t>1,00 SV ACRONIS Cyber Protect Cloud</t>
+  </si>
+  <si>
+    <t>HOWBE</t>
+  </si>
+  <si>
+    <t>03.899.222/0001-86</t>
+  </si>
+  <si>
+    <t>ESYWOLD SISTEMAS E INFORMATICA LTDA</t>
+  </si>
+  <si>
+    <t>2025-427</t>
+  </si>
+  <si>
+    <t>BOLETO.pdf</t>
+  </si>
+  <si>
+    <t>NF 037912.pdf</t>
   </si>
 </sst>
 </file>
@@ -106,9 +109,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="mm/yyyy"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -129,12 +132,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
@@ -179,30 +176,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -551,7 +542,8 @@
     <col min="11" max="11" width="14.85546875" customWidth="1"/>
     <col min="12" max="12" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="34.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -606,20 +598,20 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="9" t="s">
+      <c r="A2" s="6" t="s">
         <v>21</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>23</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="8">
-        <v>367</v>
+      <c r="E2" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="F2" s="3">
         <v>46113</v>
@@ -630,26 +622,29 @@
       <c r="H2" s="4">
         <v>46113</v>
       </c>
-      <c r="I2" s="3">
-        <v>46119</v>
+      <c r="I2" s="8">
+        <v>46127</v>
       </c>
       <c r="J2" s="3">
-        <v>46137</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" s="6">
+        <v>46142</v>
+      </c>
+      <c r="K2">
+        <v>37912</v>
+      </c>
+      <c r="L2" s="5">
         <v>1</v>
       </c>
-      <c r="M2" s="10">
-        <v>6000</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>24</v>
+      <c r="M2" s="5">
+        <v>1983.59</v>
+      </c>
+      <c r="N2" t="s">
+        <v>20</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>25</v>
+      </c>
+      <c r="P2" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>